<commit_message>
feat(crawler): complete Tiki crawler suite, full 37k records dataset, SQLite RDBMS, NoSQL, and clean team skeleton folders
</commit_message>
<xml_diff>
--- a/reports/Bang_Phan_Cong_Va_Tu_Cham_Diem.xlsx
+++ b/reports/Bang_Phan_Cong_Va_Tu_Cham_Diem.xlsx
@@ -591,9 +591,9 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>1. Xây dựng module TikiAPICrawler thu thập dữ liệu sản phẩm và bình luận.
-2. Phát triển pipeline Xử lý ngôn ngữ tự nhiên (NLP) phân tích cảm xúc tiếng Việt.
-3. Khai phá các khía cạnh đánh giá khách hàng (Aspect-based Mining: Giao hàng, Đóng gói, Chất lượng).
+          <t>1. Xây dựng module TikiAPICrawler thu thập dữ liệu sản phẩm chuẩn 35 thuộc tính và WAF solver.
+2. Xây dựng tài liệu kỹ thuật tra cứu API Tiki, danh mục Category ID và tham số truy vấn.
+3. Phân tích thị phần danh mục, phân khúc giá (Pricing Tiers) và hiệu suất thương hiệu.
 4. Thiết kế toàn bộ Slide thuyết trình báo cáo đồ án.</t>
         </is>
       </c>
@@ -627,8 +627,8 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>1. Xây dựng mô hình phân cụm khách hàng RFM và thuật toán K-Means.
-2. Phát triển Web Dashboard trực quan hóa tương tác đa chiều bằng Streamlit.
+          <t>1. Xây dựng mô hình phân cụm sản phẩm thông minh bằng K-Means (k=4).
+2. Phát triển Web Dashboard trực quan hóa tương tác sản phẩm bằng Streamlit.
 3. Giả lập luồng sự kiện Clickstream Kafka và Spark Structured Streaming.
 4. Cấu hình Docker Compose (Spark Master/Worker, Kafka, Zookeeper).
 5. Xây dựng bảng phân công và tự chấm điểm chi tiết.</t>

</xml_diff>